<commit_message>
Add login functionality with user authentication and password verification
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -441,34 +441,119 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ana</t>
+          <t>kazi</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0fb57e167b6b54d9683b86ac87f011a9</t>
+          <t>68173f916672b9772b3b901f4b24f7ec</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0f6903511de804c33a8782da55a8441b94ba5a5e087d8cd5e05d3759de4fc214</t>
+          <t>292ae84d0499d42b8f1bc229e56f7c1c099b45428c594091bd55c57f49f4e15a</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>an2</t>
+          <t>ana</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>360282fb313d4482f7427116658906e0</t>
+          <t>e91abd24b4b0af792553e0f58ce3d307</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>eb5db93de991ce61cfd7f3a0c97cdde7a08557ade3373e42e38eb22afc2eedb4</t>
+          <t>fc8843da6abcc95f4a4c46132998a17e0a4a04a277904317792481886af6a251</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>kawa</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>d7891a135350bac68491bafc28e559cb</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>9c9cac5107ddb8154057737eaa3b19a8bcf9544ebf2f8b6aaba0c5d3d87ef73a</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>_kin</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1ecac6f926e2121141e1ef19c0ec3074</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0aee650b04bded8ea3a33e14a509a418e389e3cbba9a96b02a606dcdcca2a3b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>_adria</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8514a250dc66d8f9553dc2f456781abc</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ad6b1a1dd11078396a3c4a63185f0b79341b7c0fa84717ca5fde47dd8e7c4abc</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>zod</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3ebf90816271eb651fc0c45acc09dc90</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0fffb24be289ddf35f3023d4b2ff024e2c3013f62e5f2f8022f122cdbfe53c14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>fabio</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>37db0d7216896145e975b9078258b3a7</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ab921e5dc1fce3cddddc9fcfad3087e16c167dcbb85679698e4d1af886a5b137</t>
         </is>
       </c>
     </row>

</xml_diff>